<commit_message>
Momentum scan results 2026-09-10
</commit_message>
<xml_diff>
--- a/results/momentum_failcodes_latest.xlsx
+++ b/results/momentum_failcodes_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A330"/>
+  <dimension ref="A1:A309"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -433,7 +433,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ABAT</t>
+          <t>ACDC</t>
         </is>
       </c>
     </row>
@@ -447,833 +447,833 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BHFAO</t>
+          <t>AMST</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ADAMH</t>
+          <t>ANGX</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ABUS</t>
+          <t>ACIU</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AVBP</t>
+          <t>AVX</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BLNE</t>
+          <t>ARQ</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ADAMI</t>
+          <t>ANNA</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ACDC</t>
+          <t>ACNB</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AVX</t>
+          <t>BMM</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BORR</t>
+          <t>BIRD</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AEYE</t>
+          <t>ACT</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ACET</t>
+          <t>BUR</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>BNKK</t>
+          <t>BLNE</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>AIRTP</t>
+          <t>ARLP</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ACIU</t>
+          <t>ADAMK</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CELC</t>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CLGN</t>
+          <t>ASBP</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ACU</t>
+          <t>ADAMN</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CEPU</t>
+          <t>DIBS</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>DLXY</t>
+          <t>CEPU</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AMPH</t>
+          <t>ATKR</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ADAMK</t>
+          <t>ADIL</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CHSCP</t>
+          <t>FCBM</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>FXHO</t>
+          <t>DLXY</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ANGX</t>
+          <t>ATLO</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>AFRI</t>
+          <t>AMR</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ENGN</t>
+          <t>LENZ</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>GOSS</t>
+          <t>DUKRW</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ANL</t>
+          <t>ATTO</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ALIS</t>
+          <t>APRE</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>FCUV</t>
+          <t>LFMDP</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>LBTYK</t>
+          <t>DXR</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ANNA</t>
+          <t>AVAH</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ALVO</t>
+          <t>ARTW</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>HNRG</t>
+          <t>LSTA</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>LSTA</t>
+          <t>FXHO</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ANTX</t>
+          <t>AVIR</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ALXO</t>
+          <t>ASND</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>INTR</t>
+          <t>NATH</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>NCPL</t>
+          <t>GRI</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ARLP</t>
+          <t>BFC</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>AMAN</t>
+          <t>ASTL</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>LBTYA</t>
+          <t>PASG</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>OFRM</t>
+          <t>HERE</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ARTNA</t>
+          <t>BGC</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>APRE</t>
+          <t>ATLCL</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>LFMDP</t>
+          <t>LPCN</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>PETZ</t>
+          <t>BLSM</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ATRA</t>
+          <t>AUGO</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>AQST</t>
+          <t>RGC</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>PSIG</t>
+          <t>BPAC</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ATRC</t>
+          <t>AYA</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>SNDX</t>
+          <t>WW</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ATTO</t>
+          <t>MCRB</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ATKR</t>
+          <t>BPRN</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>SKIN</t>
+          <t>BANX</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>AVAH</t>
+          <t>OPTU</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>BANX</t>
+          <t>BRLT</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>SUIG</t>
+          <t>BCAL</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>SSM</t>
+          <t>PLCE</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>BCDA</t>
+          <t>BRR</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>BAFN</t>
+          <t>BCCQ</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>BDSX</t>
+          <t>PPBT</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>BEAG</t>
+          <t>BRRWW</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>BHFAM</t>
+          <t>BCCQU</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>BEEP</t>
+          <t>RNTX</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>BHFAP</t>
+          <t>BSEM</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>BHFAN</t>
+          <t>BCCQW</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>BIVI</t>
+          <t>RTACW</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>BLSM</t>
+          <t>BSIN</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>BMM</t>
+          <t>BDCI</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>BMNP</t>
+          <t>TONX</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>BNC</t>
+          <t>BSRR</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>BMRA</t>
+          <t>BDSX</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>BOSC</t>
+          <t>BYFC</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>BPYPM</t>
+          <t>BLTE</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>BOTJ</t>
+          <t>CAC</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>BOXL</t>
+          <t>BMNP</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>BPYPN</t>
+          <t>CCNE</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>BVC</t>
+          <t>BPYPN</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>BRR</t>
+          <t>CDLR</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAAS</t>
+          <t>BPYPO</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>BRRWW</t>
+          <t>CDNA</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CABA</t>
+          <t>BRLS</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>BTBD</t>
+          <t>CDZI</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CFBK</t>
+          <t>BSBR</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CHCI</t>
+          <t>CFFN</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>BTGO</t>
+          <t>BTCT</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CHSCN</t>
+          <t>CHCI</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>BUUU</t>
+          <t>CHRD</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CHSCO</t>
+          <t>BUUU</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CDZI</t>
+          <t>BVC</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CHTRP</t>
+          <t>CLMT</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CNR</t>
+          <t>CBAT</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CHA</t>
+          <t>CLST</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CRDL</t>
+          <t>CBFV</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CLMT</t>
+          <t>CMCO</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CRESY</t>
+          <t>CBIO</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>CLST</t>
+          <t>CNR</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>CTNM</t>
+          <t>CGAU</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>CNSP</t>
+          <t>CNXC</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>CUB</t>
+          <t>CGBD</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>CNXC</t>
+          <t>COCP</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>CWST</t>
+          <t>CHCO</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>COPR</t>
+          <t>CRDL</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>DJCO</t>
+          <t>CHMG</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>DMC</t>
+          <t>CTKB</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>CRBP</t>
+          <t>CNXN</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>DMLP</t>
+          <t>CTOR</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>CRDF</t>
+          <t>COFS</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>DSC</t>
+          <t>CWBC</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>CRMD</t>
+          <t>DMC</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>EBON</t>
+          <t>DAAQ</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>CTOR</t>
+          <t>DSP</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>EEIQ</t>
+          <t>DAVE</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>ELLA</t>
+          <t>ECCU</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>DCH</t>
+          <t>DCOM</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>EPSN</t>
+          <t>EDRY</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>DERM</t>
+          <t>DDI</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>ETSS</t>
+          <t>EEIQ</t>
         </is>
       </c>
     </row>
@@ -1287,21 +1287,21 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>FLXS</t>
+          <t>EHLD</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>DLPN</t>
+          <t>DLTH</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>FLYE</t>
+          <t>FCFS</t>
         </is>
       </c>
     </row>
@@ -1315,1414 +1315,1267 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>FRNM</t>
+          <t>FMNB</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>DSGN</t>
+          <t>DMLP</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>FSEA</t>
+          <t>FRAF</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>DYNC</t>
+          <t>FSUN</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>FWAC</t>
+          <t>DOMO</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>EHLD</t>
+          <t>DPRO</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>FWDI</t>
+          <t>GRAL</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>ENSC</t>
+          <t>DRTS</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>GECC</t>
+          <t>GSM</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>EROK</t>
+          <t>ELLA</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>GITS</t>
+          <t>GTEC</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>FCNCN</t>
+          <t>ENSC</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>EOSEW</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>FLGT</t>
+          <t>HBT</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>GOAI</t>
+          <t>EPRX</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>GRAL</t>
+          <t>HPK</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>HBANM</t>
+          <t>EZPW</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>GRNQ</t>
+          <t>HSCS</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>HOWL</t>
+          <t>FBIZ</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>GSHR</t>
+          <t>HSLV</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>HTO</t>
+          <t>FBLA</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>GSM</t>
+          <t>HWBK</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>IFRX</t>
+          <t>FDSB</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>GTEC</t>
+          <t>FISI</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>IKT</t>
+          <t>FMBH</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>INBKZ</t>
+          <t>IRD</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>HCKT</t>
+          <t>FRD</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>INTG</t>
+          <t>ISTR</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>HITI</t>
+          <t>FRNM</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>INTZ</t>
+          <t>FTAIM</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>HSCS</t>
+          <t>KGEI</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>KGEI</t>
+          <t>LSBK</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>HSTM</t>
+          <t>GHXI</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>KRAQ</t>
+          <t>MDGL</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>HTT</t>
+          <t>GOAI</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>LMNR</t>
+          <t>MDXG</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>LUCY</t>
+          <t>HCM</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>IDAI</t>
+          <t>MEOH</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>MELI</t>
+          <t>HGBL</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>IMPP</t>
+          <t>HNRG</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>MGRT</t>
+          <t>MNOV</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>INMB</t>
+          <t>HNST</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>MOVE</t>
+          <t>MTC</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>IOND</t>
+          <t>NBBK</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>MSBIP</t>
+          <t>HSDT</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>IPM</t>
+          <t>NEOG</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>IRTC</t>
+          <t>HYPD</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>MWYN</t>
+          <t>NEXT</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>IVA</t>
+          <t>IKT</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>NCI</t>
+          <t>NUTX</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>JMSB</t>
+          <t>IMOS</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>NEO</t>
+          <t>NWBI</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>NEOV</t>
+          <t>IMPP</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>KRYS</t>
+          <t>OBT</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>NEWTI</t>
+          <t>INBK</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>LBRX</t>
+          <t>OCCIN</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>NEXT</t>
+          <t>INTG</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>LIFE</t>
+          <t>OCUL</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>NSAIU</t>
+          <t>ITIC</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>LNSR</t>
+          <t>OGC</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>NSTS</t>
+          <t>JAN</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>LSBK</t>
+          <t>OMER</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>LTGO</t>
+          <t>JANX</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>MDXG</t>
+          <t>ORIO</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>NVNO</t>
+          <t>KRAQ</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>PAYO</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>NXTC</t>
+          <t>KRNY</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>METCZ</t>
+          <t>PAYP</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>OABI</t>
+          <t>LCLN</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>MLYS</t>
+          <t>PBLS</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>OMER</t>
+          <t>LINK</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>MNOV</t>
+          <t>PBM</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>OMSE</t>
+          <t>MBNKO</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>MNSB</t>
+          <t>PKBK</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>ONBPO</t>
+          <t>MBWM</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>MNTK</t>
+          <t>PLMR</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>ORIO</t>
+          <t>MCGA</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>MTC</t>
+          <t>PPIH</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>OXLC</t>
+          <t>MGRT</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>MTLS</t>
+          <t>PRME</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>OXLCG</t>
+          <t>MKTX</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>NEOG</t>
+          <t>PROK</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>OXLCZ</t>
+          <t>MSBI</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>NKTX</t>
+          <t>PRTS</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>PAHC</t>
+          <t>MSBIP</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>NTRB</t>
+          <t>RIBB</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>PCAPU</t>
+          <t>RNW</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>NTWOW</t>
+          <t>RYM</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>PCRX</t>
+          <t>NEO</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>NVA</t>
+          <t>SAFT</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>PESI</t>
+          <t>NEWTI</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>PLCE</t>
+          <t>SCZM</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>NXB</t>
+          <t>NTRA</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>PRHI</t>
+          <t>SLDE</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>OCCIN</t>
+          <t>NTRB</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>OESX</t>
+          <t>STEP</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>PTN</t>
+          <t>SUNC</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>ONBPP</t>
+          <t>NVCT</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>QNBC</t>
+          <t>TDAC</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>OPCH</t>
+          <t>TELA</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>QNRX</t>
+          <t>OHAC</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>ORBS</t>
+          <t>TJGC</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>RECT</t>
+          <t>TLX</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>OXLCI</t>
+          <t>ONCHU</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>OPCH</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>RILYN</t>
+          <t>TTRX</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>RILYZ</t>
+          <t>OSBC</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>PAYP</t>
+          <t>VOXR</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>RNGT</t>
+          <t>OTAI</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>PBAM</t>
+          <t>WHK</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>RTAC</t>
+          <t>OXLCG</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>PBLS</t>
+          <t>XIIIU</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>PDLB</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>PBM</t>
+          <t>PFIS</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>SAIH</t>
+          <t>PFLA</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>PCVX</t>
+          <t>PGY</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>SAX</t>
+          <t>PLBC</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>PECE</t>
+          <t>PLUS</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>SCATU</t>
+          <t>PMVP</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>PEPG</t>
+          <t>PRZO</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>SCTX</t>
+          <t>PTN</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>PLGO</t>
+          <t>PVLA</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>SIEB</t>
+          <t>QNRX</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>PLSE</t>
+          <t>QRVO</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>SLAB</t>
+          <t>RANI</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>PMTS</t>
+          <t>RCEL</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>SLDB</t>
+          <t>RGLD</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>PPHC</t>
+          <t>RHLD</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>SLMBP</t>
+          <t>RILYG</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>PPIH</t>
+          <t>RRBI</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>RWAYI</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>SND</t>
+          <t>SAIH</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>PRTS</t>
+          <t>SATA</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>QRVO</t>
+          <t>SBFG</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>STRK</t>
+          <t>SCSC</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>RANI</t>
+          <t>SGP</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>SVRN</t>
+          <t>SKYX</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>RBKB</t>
+          <t>SLAB</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>SWVL</t>
+          <t>SLDB</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>RCEL</t>
+          <t>SND</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>TELA</t>
+          <t>SPFI</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>RFAMU</t>
+          <t>STKE</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>TGTX</t>
+          <t>STRD</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>RILYT</t>
+          <t>SVRN</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>TIL</t>
+          <t>SWVL</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>RRBI</t>
+          <t>TAOX</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>TJGC</t>
+          <t>TARS</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>SAFT</t>
+          <t>TCBX</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>TLF</t>
+          <t>TGHL</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>SATA</t>
+          <t>TII</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>TOP</t>
+          <t>TLF</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>SBC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>TORO</t>
+          <t>TRNZ</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>SCWO</t>
+          <t>USAU</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>VAI</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>SDGR</t>
+          <t>NVA</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>TRNZ</t>
+          <t>SECZ</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>SENEA</t>
+          <t>DH</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>SFBC</t>
+          <t>NXTC</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>SGP</t>
+          <t>RDI</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>SLDE</t>
+          <t>BTGO</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>SLDP</t>
+          <t>NEOV</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>SLN</t>
+          <t>BIXIW</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>SMCIP</t>
+          <t>MNTK</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>SMTI</t>
+          <t>OYSER</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>SNDL</t>
+          <t>TITN</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>SPRB</t>
+          <t>NUAI</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>SUNC</t>
+          <t>ALT</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>TDAC</t>
+          <t>ORBS</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>TH</t>
+          <t>BBBYW</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>TIGO</t>
+          <t>MLYS</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>TRLV</t>
+          <t>DAAQU</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>TTRX</t>
+          <t>LHAI</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>VOR</t>
+          <t>BTBD</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>WSBCO</t>
+          <t>ATRA</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>TITN</t>
+          <t>XTERW</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>AKTX</t>
+          <t>DGICB</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>AACPR</t>
+          <t>KPLT</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>MMED</t>
+          <t>SCWO</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>NDRA</t>
+          <t>PXS</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>JANX</t>
-        </is>
-      </c>
-    </row>
-    <row r="310">
-      <c r="A310" t="inlineStr">
-        <is>
-          <t>DPRO</t>
-        </is>
-      </c>
-    </row>
-    <row r="311">
-      <c r="A311" t="inlineStr">
-        <is>
-          <t>AGBK</t>
-        </is>
-      </c>
-    </row>
-    <row r="312">
-      <c r="A312" t="inlineStr">
-        <is>
-          <t>OFS</t>
-        </is>
-      </c>
-    </row>
-    <row r="313">
-      <c r="A313" t="inlineStr">
-        <is>
-          <t>TARS</t>
-        </is>
-      </c>
-    </row>
-    <row r="314">
-      <c r="A314" t="inlineStr">
-        <is>
-          <t>RCBC</t>
-        </is>
-      </c>
-    </row>
-    <row r="315">
-      <c r="A315" t="inlineStr">
-        <is>
-          <t>PYXS</t>
-        </is>
-      </c>
-    </row>
-    <row r="316">
-      <c r="A316" t="inlineStr">
-        <is>
-          <t>ASND</t>
-        </is>
-      </c>
-    </row>
-    <row r="317">
-      <c r="A317" t="inlineStr">
-        <is>
-          <t>CBIO</t>
-        </is>
-      </c>
-    </row>
-    <row r="318">
-      <c r="A318" t="inlineStr">
-        <is>
-          <t>MCRB</t>
-        </is>
-      </c>
-    </row>
-    <row r="319">
-      <c r="A319" t="inlineStr">
-        <is>
-          <t>USDEW</t>
-        </is>
-      </c>
-    </row>
-    <row r="320">
-      <c r="A320" t="inlineStr">
-        <is>
-          <t>PROK</t>
-        </is>
-      </c>
-    </row>
-    <row r="321">
-      <c r="A321" t="inlineStr">
-        <is>
-          <t>ADIL</t>
-        </is>
-      </c>
-    </row>
-    <row r="322">
-      <c r="A322" t="inlineStr">
-        <is>
-          <t>BMEA</t>
-        </is>
-      </c>
-    </row>
-    <row r="323">
-      <c r="A323" t="inlineStr">
-        <is>
-          <t>DFDV</t>
-        </is>
-      </c>
-    </row>
-    <row r="324">
-      <c r="A324" t="inlineStr">
-        <is>
-          <t>SPWH</t>
-        </is>
-      </c>
-    </row>
-    <row r="325">
-      <c r="A325" t="inlineStr">
-        <is>
-          <t>PXS</t>
-        </is>
-      </c>
-    </row>
-    <row r="326">
-      <c r="A326" t="inlineStr">
-        <is>
-          <t>RDI</t>
-        </is>
-      </c>
-    </row>
-    <row r="327">
-      <c r="A327" t="inlineStr">
-        <is>
-          <t>DH</t>
-        </is>
-      </c>
-    </row>
-    <row r="328">
-      <c r="A328" t="inlineStr">
-        <is>
-          <t>INO</t>
-        </is>
-      </c>
-    </row>
-    <row r="329">
-      <c r="A329" t="inlineStr">
-        <is>
-          <t>FTH</t>
-        </is>
-      </c>
-    </row>
-    <row r="330">
-      <c r="A330" t="inlineStr">
-        <is>
-          <t>AGIG</t>
+          <t>SIEB</t>
         </is>
       </c>
     </row>

</xml_diff>